<commit_message>
schreiben... winkelerkennung mit mediapipe mit 45°
</commit_message>
<xml_diff>
--- a/armwinkel auswertung/armwinkel mediapipe world.xlsx
+++ b/armwinkel auswertung/armwinkel mediapipe world.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ampelman\Desktop\Masterarbeit\armwinkel auswertung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A21B09F-5308-4104-9E32-7EFEEE97D423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A88BE7-64B3-4932-B61C-141D539E471E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4B6C38A1-A2E0-47AD-A4A2-CC2594FC12BF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="25">
   <si>
     <t>referenze achse</t>
   </si>
@@ -93,6 +93,27 @@
   </si>
   <si>
     <t>total diff</t>
+  </si>
+  <si>
+    <t>Kameraneigung</t>
+  </si>
+  <si>
+    <t>Winkelpunkt</t>
+  </si>
+  <si>
+    <t>Referenzachse</t>
+  </si>
+  <si>
+    <t>Schultermitte</t>
+  </si>
+  <si>
+    <t>Schulter</t>
+  </si>
+  <si>
+    <t>0°</t>
+  </si>
+  <si>
+    <t>32,5°</t>
   </si>
 </sst>
 </file>
@@ -140,7 +161,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -148,17 +169,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -493,22 +531,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECEC828-14DB-4FFC-B0C6-765AB77059C1}">
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:X30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" customWidth="1"/>
     <col min="15" max="15" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -603,50 +640,50 @@
       </c>
     </row>
     <row r="3" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
+      <c r="A3">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3">
         <v>88</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3">
         <v>81</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3">
         <v>49</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3">
         <v>63</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3">
         <v>-6</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3">
         <v>-14</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5">
+      <c r="J3"/>
+      <c r="K3">
         <f t="shared" ref="K3:K13" si="0">SUM(D3,E3)/2 -90</f>
         <v>-5.5</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5">
+      <c r="L3"/>
+      <c r="M3">
         <f t="shared" ref="M3:M13" si="1">SUM(F3,G3)/2 -45</f>
         <v>11</v>
       </c>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5">
+      <c r="N3"/>
+      <c r="O3">
         <f t="shared" ref="O3:O13" si="2">SUM(H3,I3)/2</f>
         <v>-10</v>
       </c>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5">
+      <c r="P3"/>
+      <c r="Q3">
         <f t="shared" ref="Q3:Q13" si="3">(ABS(K3)+ABS(M3)+ABS(O3))/3</f>
         <v>8.8333333333333339</v>
       </c>
@@ -749,99 +786,91 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+      <c r="A6">
         <v>32.5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6">
         <v>85</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6">
         <v>78</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6">
         <v>85</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6">
         <v>73</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6">
         <v>32</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6">
         <v>20</v>
       </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5">
+      <c r="K6">
         <f t="shared" si="0"/>
         <v>-8.5</v>
       </c>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5">
+      <c r="M6">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5">
+      <c r="O6">
         <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5">
+      <c r="Q6">
         <f t="shared" si="3"/>
         <v>22.833333333333332</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+      <c r="A7">
         <v>32.5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7">
         <v>85</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7">
         <v>78</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7">
         <v>85</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7">
         <v>73</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7">
         <v>-32</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7">
         <v>-20</v>
       </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5">
+      <c r="K7">
         <f t="shared" si="0"/>
         <v>-8.5</v>
       </c>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5">
+      <c r="M7">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5">
+      <c r="O7">
         <f t="shared" si="2"/>
         <v>-26</v>
       </c>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5">
+      <c r="Q7">
         <f t="shared" si="3"/>
         <v>22.833333333333332</v>
       </c>
@@ -990,50 +1019,46 @@
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11">
         <v>86</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11">
         <v>80</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11">
         <v>59</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11">
         <v>60</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11">
         <v>-13</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11">
         <v>-10</v>
       </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5">
+      <c r="K11">
         <f t="shared" si="0"/>
         <v>-7</v>
       </c>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5">
+      <c r="M11">
         <f t="shared" si="1"/>
         <v>14.5</v>
       </c>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5">
+      <c r="O11">
         <f t="shared" si="2"/>
         <v>-11.5</v>
       </c>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5">
+      <c r="Q11">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
@@ -1128,7 +1153,418 @@
         <v>18.333333333333332</v>
       </c>
     </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22" s="5"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="6">
+        <v>92</v>
+      </c>
+      <c r="E23" s="6">
+        <v>81</v>
+      </c>
+      <c r="F23" s="6">
+        <v>49</v>
+      </c>
+      <c r="G23" s="6">
+        <v>63</v>
+      </c>
+      <c r="H23" s="6">
+        <v>6</v>
+      </c>
+      <c r="I23" s="6">
+        <v>14</v>
+      </c>
+      <c r="J23" s="6">
+        <f>SUM(D23,E23)/2 -90</f>
+        <v>-3.5</v>
+      </c>
+      <c r="K23" s="6">
+        <f>SUM(F23,G23)/2 -45</f>
+        <v>11</v>
+      </c>
+      <c r="L23" s="6">
+        <f>SUM(H23,I23)/2</f>
+        <v>10</v>
+      </c>
+      <c r="M23" s="6">
+        <f>(ABS(J23)+ABS(K23)+ABS(L23))/3</f>
+        <v>8.1666666666666661</v>
+      </c>
+      <c r="N23" s="6"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="5">
+        <v>88</v>
+      </c>
+      <c r="E24" s="5">
+        <v>81</v>
+      </c>
+      <c r="F24" s="5">
+        <v>49</v>
+      </c>
+      <c r="G24" s="5">
+        <v>63</v>
+      </c>
+      <c r="H24" s="5">
+        <v>-6</v>
+      </c>
+      <c r="I24" s="5">
+        <v>-14</v>
+      </c>
+      <c r="J24" s="5">
+        <f>SUM(D24,E24)/2 -90</f>
+        <v>-5.5</v>
+      </c>
+      <c r="K24" s="5">
+        <f>SUM(F24,G24)/2 -45</f>
+        <v>11</v>
+      </c>
+      <c r="L24" s="5">
+        <f>SUM(H24,I24)/2</f>
+        <v>-10</v>
+      </c>
+      <c r="M24" s="5">
+        <f>(ABS(J24)+ABS(K24)+ABS(L24))/3</f>
+        <v>8.8333333333333339</v>
+      </c>
+      <c r="N24" s="5"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="5">
+        <v>81</v>
+      </c>
+      <c r="E25" s="5">
+        <v>75</v>
+      </c>
+      <c r="F25" s="5">
+        <v>50</v>
+      </c>
+      <c r="G25" s="5">
+        <v>64</v>
+      </c>
+      <c r="H25" s="5">
+        <v>5</v>
+      </c>
+      <c r="I25" s="5">
+        <v>3</v>
+      </c>
+      <c r="J25" s="5">
+        <f>SUM(D25,E25)/2 -90</f>
+        <v>-12</v>
+      </c>
+      <c r="K25" s="5">
+        <f>SUM(F25,G25)/2 -45</f>
+        <v>12</v>
+      </c>
+      <c r="L25" s="5">
+        <f>SUM(H25,I25)/2</f>
+        <v>4</v>
+      </c>
+      <c r="M25" s="5">
+        <f>(ABS(J25)+ABS(K25)+ABS(L25))/3</f>
+        <v>9.3333333333333339</v>
+      </c>
+      <c r="N25" s="5"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="5">
+        <v>90</v>
+      </c>
+      <c r="E26" s="5">
+        <v>84</v>
+      </c>
+      <c r="F26" s="5">
+        <v>59</v>
+      </c>
+      <c r="G26" s="5">
+        <v>73</v>
+      </c>
+      <c r="H26" s="5">
+        <v>15</v>
+      </c>
+      <c r="I26" s="5">
+        <v>12</v>
+      </c>
+      <c r="J26" s="5">
+        <f>SUM(D26,E26)/2 -90</f>
+        <v>-3</v>
+      </c>
+      <c r="K26" s="5">
+        <f>SUM(F26,G26)/2 -45</f>
+        <v>21</v>
+      </c>
+      <c r="L26" s="5">
+        <f>SUM(H26,I26)/2</f>
+        <v>13.5</v>
+      </c>
+      <c r="M26" s="5">
+        <f>(ABS(J26)+ABS(K26)+ABS(L26))/3</f>
+        <v>12.5</v>
+      </c>
+      <c r="N26" s="5"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="7">
+        <v>86</v>
+      </c>
+      <c r="E27" s="7">
+        <v>80</v>
+      </c>
+      <c r="F27" s="7">
+        <v>59</v>
+      </c>
+      <c r="G27" s="7">
+        <v>60</v>
+      </c>
+      <c r="H27" s="7">
+        <v>13</v>
+      </c>
+      <c r="I27" s="7">
+        <v>10</v>
+      </c>
+      <c r="J27" s="7">
+        <f>SUM(D27,E27)/2 -90</f>
+        <v>-7</v>
+      </c>
+      <c r="K27" s="7">
+        <f>SUM(F27,G27)/2 -45</f>
+        <v>14.5</v>
+      </c>
+      <c r="L27" s="7">
+        <f>SUM(H27,I27)/2</f>
+        <v>11.5</v>
+      </c>
+      <c r="M27" s="7">
+        <f>(ABS(J27)+ABS(K27)+ABS(L27))/3</f>
+        <v>11</v>
+      </c>
+      <c r="N27" s="7"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="5">
+        <v>86</v>
+      </c>
+      <c r="E28" s="5">
+        <v>80</v>
+      </c>
+      <c r="F28" s="5">
+        <v>59</v>
+      </c>
+      <c r="G28" s="5">
+        <v>60</v>
+      </c>
+      <c r="H28" s="5">
+        <v>-13</v>
+      </c>
+      <c r="I28" s="5">
+        <v>-10</v>
+      </c>
+      <c r="J28" s="5">
+        <f>SUM(D28,E28)/2 -90</f>
+        <v>-7</v>
+      </c>
+      <c r="K28" s="5">
+        <f>SUM(F28,G28)/2 -45</f>
+        <v>14.5</v>
+      </c>
+      <c r="L28" s="5">
+        <f>SUM(H28,I28)/2</f>
+        <v>-11.5</v>
+      </c>
+      <c r="M28" s="5">
+        <f>(ABS(J28)+ABS(K28)+ABS(L28))/3</f>
+        <v>11</v>
+      </c>
+      <c r="N28" s="5"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="5">
+        <v>91</v>
+      </c>
+      <c r="E29" s="5">
+        <v>91</v>
+      </c>
+      <c r="F29" s="5">
+        <v>76</v>
+      </c>
+      <c r="G29" s="5">
+        <v>73</v>
+      </c>
+      <c r="H29" s="5">
+        <v>29</v>
+      </c>
+      <c r="I29" s="5">
+        <v>20</v>
+      </c>
+      <c r="J29" s="5">
+        <f>SUM(D29,E29)/2 -90</f>
+        <v>1</v>
+      </c>
+      <c r="K29" s="5">
+        <f>SUM(F29,G29)/2 -45</f>
+        <v>29.5</v>
+      </c>
+      <c r="L29" s="5">
+        <f>SUM(H29,I29)/2</f>
+        <v>24.5</v>
+      </c>
+      <c r="M29" s="5">
+        <f>(ABS(J29)+ABS(K29)+ABS(L29))/3</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="N29" s="5"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5">
+        <v>89</v>
+      </c>
+      <c r="E30" s="5">
+        <v>89</v>
+      </c>
+      <c r="F30" s="5">
+        <v>76</v>
+      </c>
+      <c r="G30" s="5">
+        <v>73</v>
+      </c>
+      <c r="H30" s="5">
+        <v>29</v>
+      </c>
+      <c r="I30" s="5">
+        <v>20</v>
+      </c>
+      <c r="J30" s="5">
+        <f>SUM(D30,E30)/2 -90</f>
+        <v>-1</v>
+      </c>
+      <c r="K30" s="5">
+        <f>SUM(F30,G30)/2 -45</f>
+        <v>29.5</v>
+      </c>
+      <c r="L30" s="5">
+        <f>SUM(H30,I30)/2</f>
+        <v>24.5</v>
+      </c>
+      <c r="M30" s="5">
+        <f>(ABS(J30)+ABS(K30)+ABS(L30))/3</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="N30" s="5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>